<commit_message>
update ppt y tarea 3
</commit_message>
<xml_diff>
--- a/presentaciones.xlsx
+++ b/presentaciones.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e2f577dda2fcbe77/Documentos/LAB-MAA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanc\OneDrive\Documentos\LAB-MAA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{92B3A7D9-A9C9-4183-84C8-8767C1D8C6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DF55DD9-54FB-4A67-B51D-CD9714404E71}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E7FBF5-9263-4D5D-8381-6C7B972C65A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -607,17 +607,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -645,6 +637,17 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -964,645 +967,645 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:7" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="6" t="s">
+      <c r="G2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A3" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A4" s="9" t="s">
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A4" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A5" s="6" t="s">
+      <c r="G4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A5" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="D5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="6" t="s">
+      <c r="G5" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="6" t="s">
+      <c r="D6" s="4"/>
+      <c r="E6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:7" s="16" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A7" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="18" t="s">
+      <c r="D7" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A8" t="s">
+      <c r="G7" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A8" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D8" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="G8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A9" t="s">
+      <c r="G8" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="16" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A9" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="D9" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A10" t="s">
+      <c r="G9" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A10" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="D10" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="A11" t="s">
+      <c r="G10" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="16" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A11" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="D11" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A12" t="s">
+      <c r="G11" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A12" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="D12" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="G12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A13" t="s">
+      <c r="G12" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A13" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="D13" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="G13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A14" s="6" t="s">
+      <c r="G13" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A14" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="9" t="s">
+      <c r="D14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A15" s="6" t="s">
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A15" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="6" t="s">
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G15" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A16" s="6" t="s">
+      <c r="G15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A16" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="6" t="s">
+      <c r="D16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A17" s="6" t="s">
+      <c r="G16" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A17" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="D17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A18" s="6" t="s">
+      <c r="G17" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A18" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="D18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="6" t="s">
+      <c r="G18" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="6" t="s">
+      <c r="D19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A20" s="6" t="s">
+      <c r="G19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="6" t="s">
+      <c r="D20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G20" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A21" s="6" t="s">
+      <c r="G20" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="9" t="s">
+      <c r="D21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A22" s="6" t="s">
+      <c r="G21" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="2" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A22" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="6" t="s">
+      <c r="D22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A23" s="6" t="s">
+      <c r="G22" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A23" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="9" t="s">
+      <c r="D23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" s="6" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A24" s="6" t="s">
+      <c r="G23" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A24" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="9" t="s">
+      <c r="D24" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G24" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A25" s="6" t="s">
+      <c r="G24" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D25" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="9" t="s">
+      <c r="D25" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" s="6" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A26" s="9" t="s">
+      <c r="G25" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="2" customFormat="1" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A26" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D26" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" s="9" t="s">
+      <c r="D26" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="F26" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="6" t="s">
+      <c r="D27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A28" s="6" t="s">
+    <row r="28" spans="1:7" s="2" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E28" s="9" t="s">
+      <c r="D28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G28" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A29" s="6" t="s">
+      <c r="G28" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E29" s="6" t="s">
+      <c r="D29" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G29" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1669,299 +1672,299 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="26.5" x14ac:dyDescent="0.75">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="8" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>